<commit_message>
case 00 with new biomass
</commit_message>
<xml_diff>
--- a/case_studies/base_case_00_5_dd/2050/technologies.xlsx
+++ b/case_studies/base_case_00_5_dd/2050/technologies.xlsx
@@ -694,7 +694,7 @@
         <v>115.42</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>452.75</v>
+        <v>453.65</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>0</v>
@@ -712,10 +712,10 @@
         <v>0</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>230.83</v>
+        <v>230.84</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>271.85</v>
+        <v>274.14</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>37.46</v>
@@ -736,7 +736,7 @@
         <v>235.42</v>
       </c>
       <c r="X2" s="3" t="n">
-        <v>0</v>
+        <v>6.85</v>
       </c>
       <c r="Y2" s="3" t="n">
         <v>0</v>
@@ -767,10 +767,10 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>0</v>
+        <v>5.21</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.39</v>
+        <v>0</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>45.66</v>
@@ -785,10 +785,10 @@
         <v>8.08</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>0.32</v>
+        <v>3.55</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>17.75</v>
+        <v>0</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>35.39</v>
@@ -885,10 +885,10 @@
         <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>186.17</v>
+        <v>448.8</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>586.37</v>
+        <v>897.77</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>20.3</v>
@@ -906,19 +906,19 @@
         <v>0</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>410</v>
+        <v>1107.98</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>445.28</v>
+        <v>1143.25</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>48.73</v>
+        <v>272.26</v>
       </c>
       <c r="S4" s="3" t="n">
         <v>43.32</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>231.42</v>
+        <v>448.8</v>
       </c>
       <c r="U4" s="3" t="n">
         <v>0</v>
@@ -927,10 +927,10 @@
         <v>11.05</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>249.55</v>
+        <v>269.25</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y4" s="3" t="n">
         <v>0</v>
@@ -985,13 +985,13 @@
         <v>108.43</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>394.04</v>
+        <v>424.14</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>148.52</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>0</v>
+        <v>100.9</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>745.4</v>
@@ -1003,34 +1003,34 @@
         <v>0</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>136.97</v>
+        <v>372.73</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>136.97</v>
+        <v>391.69</v>
       </c>
       <c r="R5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>0</v>
+        <v>12.77</v>
       </c>
       <c r="T5" s="5" t="n">
-        <v>125.97</v>
+        <v>209.33</v>
       </c>
       <c r="U5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="V5" s="5" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="W5" s="5" t="n">
-        <v>180.97</v>
+        <v>713.5</v>
       </c>
       <c r="X5" s="5" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>0</v>
+        <v>53506.64</v>
       </c>
       <c r="Z5" s="5" t="n">
         <v>204.22</v>
@@ -1061,7 +1061,7 @@
         <v>91.76000000000001</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0</v>
+        <v>347.89</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>62.79</v>
@@ -1082,37 +1082,37 @@
         <v>67.88</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>240.1</v>
+        <v>160.23</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>42.99</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0</v>
+        <v>162.15</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>565.33</v>
+        <v>179.06</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>565.33</v>
+        <v>179.06</v>
       </c>
       <c r="O6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>134.05</v>
+        <v>529.65</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>139.43</v>
+        <v>543.11</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0</v>
+        <v>63.82</v>
       </c>
       <c r="S6" s="3" t="n">
         <v>9.16</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>95.54000000000001</v>
+        <v>230.03</v>
       </c>
       <c r="U6" s="3" t="n">
         <v>0</v>
@@ -1121,10 +1121,10 @@
         <v>0</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>121.16</v>
+        <v>63.82</v>
       </c>
       <c r="X6" s="3" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y6" s="3" t="n">
         <v>0</v>
@@ -1167,7 +1167,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
@@ -1203,7 +1203,7 @@
         <v>0</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>20.61</v>
+        <v>19.77</v>
       </c>
       <c r="S7" s="5" t="n">
         <v>15.94</v>
@@ -1282,7 +1282,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0</v>
+        <v>81.45999999999999</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>136.33</v>
@@ -1294,19 +1294,19 @@
         <v>0</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>372.36</v>
+        <v>446.76</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>427.03</v>
+        <v>476.68</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>127.74</v>
+        <v>102.09</v>
       </c>
       <c r="S8" s="3" t="n">
         <v>50.33</v>
       </c>
       <c r="T8" s="3" t="n">
-        <v>136.83</v>
+        <v>218.29</v>
       </c>
       <c r="U8" s="3" t="n">
         <v>0</v>
@@ -1315,13 +1315,13 @@
         <v>1.54</v>
       </c>
       <c r="W8" s="3" t="n">
-        <v>101.67</v>
+        <v>855.89</v>
       </c>
       <c r="X8" s="3" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>0</v>
+        <v>76708.08</v>
       </c>
       <c r="Z8" s="3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
reset CO2 export limits
</commit_message>
<xml_diff>
--- a/case_studies/base_case_00_5_dd/2050/technologies.xlsx
+++ b/case_studies/base_case_00_5_dd/2050/technologies.xlsx
@@ -679,7 +679,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0</v>
@@ -694,13 +694,13 @@
         <v>114.43</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>458.64</v>
+        <v>450.45</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0</v>
+        <v>47.74</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>946.41</v>
@@ -712,10 +712,10 @@
         <v>0</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>228.86</v>
+        <v>330.31</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>279.52</v>
+        <v>382.68</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>35.44</v>
@@ -724,7 +724,7 @@
         <v>23.37</v>
       </c>
       <c r="T2" s="3" t="n">
-        <v>159.94</v>
+        <v>162.17</v>
       </c>
       <c r="U2" s="3" t="n">
         <v>0</v>
@@ -733,10 +733,10 @@
         <v>69.83</v>
       </c>
       <c r="W2" s="3" t="n">
-        <v>242.02</v>
+        <v>241.7</v>
       </c>
       <c r="X2" s="3" t="n">
-        <v>0</v>
+        <v>6.85</v>
       </c>
       <c r="Y2" s="3" t="n">
         <v>0</v>
@@ -885,19 +885,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>185.63</v>
+        <v>56.57</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>654.65</v>
+        <v>546.15</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>20.3</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0</v>
+        <v>221.92</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>1369.36</v>
+        <v>1519.72</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>1369.36</v>
@@ -906,19 +906,19 @@
         <v>0</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>408.72</v>
+        <v>584.72</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>451.24</v>
+        <v>627.24</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>48.47</v>
+        <v>0</v>
       </c>
       <c r="S4" s="3" t="n">
         <v>47.61</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>231.42</v>
+        <v>278.49</v>
       </c>
       <c r="U4" s="3" t="n">
         <v>0</v>
@@ -927,10 +927,10 @@
         <v>13.99</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>312.87</v>
+        <v>357.12</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y4" s="3" t="n">
         <v>0</v>
@@ -985,13 +985,13 @@
         <v>108.43</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>394.84</v>
+        <v>356.02</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>148.52</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>0</v>
+        <v>156.59</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>745.4</v>
@@ -1003,34 +1003,34 @@
         <v>0</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>136.2</v>
+        <v>549.62</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>136.2</v>
+        <v>561.59</v>
       </c>
       <c r="R5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="T5" s="5" t="n">
-        <v>125.97</v>
+        <v>265.02</v>
       </c>
       <c r="U5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="V5" s="5" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="W5" s="5" t="n">
-        <v>181.09</v>
+        <v>556.0599999999999</v>
       </c>
       <c r="X5" s="5" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>0</v>
+        <v>41530.27</v>
       </c>
       <c r="Z5" s="5" t="n">
         <v>204.22</v>
@@ -1070,7 +1070,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0</v>
+        <v>1.81</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>11.11</v>
@@ -1082,49 +1082,49 @@
         <v>67.83</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>240.2</v>
+        <v>174.67</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>42.99</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0</v>
+        <v>165.37</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>565.33</v>
+        <v>197.83</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>565.33</v>
+        <v>197.83</v>
       </c>
       <c r="O6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>134.02</v>
+        <v>487.08</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>139.56</v>
+        <v>508.29</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>9.42</v>
+        <v>14.27</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>95.54000000000001</v>
+        <v>233.2</v>
       </c>
       <c r="U6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>0</v>
+        <v>0.73</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>121.27</v>
+        <v>75.75</v>
       </c>
       <c r="X6" s="3" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y6" s="3" t="n">
         <v>0</v>
@@ -1176,7 +1176,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>48.52</v>
+        <v>0</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>59.3</v>
@@ -1185,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>0</v>
+        <v>35.68</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>0</v>
@@ -1203,7 +1203,7 @@
         <v>0</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>20.6</v>
+        <v>19.87</v>
       </c>
       <c r="S7" s="5" t="n">
         <v>15.89</v>
@@ -1218,13 +1218,13 @@
         <v>1.73</v>
       </c>
       <c r="W7" s="5" t="n">
-        <v>19.5</v>
+        <v>48.1</v>
       </c>
       <c r="X7" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>0</v>
+        <v>2934.72</v>
       </c>
       <c r="Z7" s="5" t="n">
         <v>0</v>
@@ -1282,7 +1282,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0</v>
+        <v>80.31999999999999</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>136.33</v>
@@ -1294,19 +1294,19 @@
         <v>0</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>372.33</v>
+        <v>460.93</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>427.03</v>
+        <v>490.77</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>128.05</v>
+        <v>102.32</v>
       </c>
       <c r="S8" s="3" t="n">
         <v>50.29</v>
       </c>
       <c r="T8" s="3" t="n">
-        <v>136.69</v>
+        <v>217.01</v>
       </c>
       <c r="U8" s="3" t="n">
         <v>0</v>
@@ -1315,13 +1315,13 @@
         <v>2.05</v>
       </c>
       <c r="W8" s="3" t="n">
-        <v>101.76</v>
+        <v>692.63</v>
       </c>
       <c r="X8" s="3" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>0</v>
+        <v>61254.54</v>
       </c>
       <c r="Z8" s="3" t="n">
         <v>0</v>

</xml_diff>